<commit_message>
sheets: format first data row, GDP cutoff by quarter, cover fixes, Allow-access note
Found by evaluating a private copy against a real refresh-data fixture:
the DATA_ROW formula cell's own style overrode the column number format,
GDP's cutoff showed only the year, and Sheets' Allow-access bar was never
mentioned to customers.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/integrations/google-sheets/Viet-Dataverse-Google-Sheets-Template.xlsx
+++ b/integrations/google-sheets/Viet-Dataverse-Google-Sheets-Template.xlsx
@@ -195,7 +195,9 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -607,11 +609,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:C15"/>
+  <dimension ref="B2:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
     <col width="70" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -674,65 +676,77 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Mở tab "Tổng quan" để xem bảng tổng quan; chín tab sau là dữ liệu chi tiết, mỗi tab có biểu đồ.</t>
+          <t>Mở tab "Tổng quan" để xem bảng tổng quan; chín tab sau là dữ liệu chi tiết, biểu đồ nằm ở tab Tổng quan.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1">
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Chưa có key?</t>
+          <t>Thấy thanh vàng?</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Lấy miễn phí tại https://vietdataverse.online/pages/developer.html</t>
+          <t>Sheets hỏi "Allow access" / "Cho phép truy cập" ở đầu trang: bấm cho phép, nếu không file không lấy được dữ liệu.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1">
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Làm mới</t>
+          <t>Chưa có key?</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Tăng số ở ô C7 (1 → 2 → 3…). Tải lại trang KHÔNG làm mới — Google giữ cache ~1 giờ.</t>
+          <t>Lấy miễn phí tại https://vietdataverse.online/pages/developer.html</t>
         </is>
       </c>
     </row>
     <row r="13" ht="32" customHeight="1">
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Khoảng thời gian</t>
+          <t>Làm mới</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Chọn ở ô C8: 1m (1 tháng), 1y (1 năm), all (toàn bộ lịch sử).</t>
+          <t>Tăng số ở ô C7 (1 → 2 → 3…). Tải lại trang KHÔNG làm mới — Google giữ cache ~1 giờ.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1">
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Hạn mức</t>
+          <t>Khoảng thời gian</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Cả file chỉ tốn 1 lượt API mỗi lần làm mới (không phải 9). Miễn phí 20 lượt/tháng; gói trả phí 1.000 lượt/tháng.</t>
+          <t>Chọn ở ô C8: 1m (1 tháng), 1y (1 năm), all (toàn bộ lịch sử).</t>
         </is>
       </c>
     </row>
     <row r="15" ht="32" customHeight="1">
       <c r="B15" s="6" t="inlineStr">
         <is>
+          <t>Hạn mức</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Cả file chỉ tốn 1 lượt API mỗi lần làm mới (không phải 9). Miễn phí 20 lượt/tháng; gói trả phí 1.000 lượt/tháng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="32" customHeight="1">
+      <c r="B16" s="6" t="inlineStr">
+        <is>
           <t>Bảo mật</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C16" s="7" t="inlineStr">
         <is>
           <t>Key nằm trong ô C6 của bản copy của bạn. Đừng chia sẻ file này cho người lạ.</t>
         </is>
@@ -759,7 +773,7 @@
   <cols>
     <col width="13" customWidth="1" style="30" min="1" max="1"/>
     <col width="13" customWidth="1" style="30" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" style="27" min="4" max="4"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
@@ -779,7 +793,7 @@
         </is>
       </c>
       <c r="B2" s="25">
-        <f>IF(VDV_STATUS&lt;&gt;"dataset", "—", IFERROR(INDEX(A6:A2500, COUNTA(A6:A2500)), "—"))</f>
+        <f>IF(VDV_STATUS&lt;&gt;"dataset", "—", IFERROR(INDEX(H6:H2500, COUNTA(H6:H2500)), "—"))</f>
         <v/>
       </c>
     </row>
@@ -816,11 +830,11 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6">
+      <c r="A6" s="30">
         <f>IF(VDV_STATUS&lt;&gt;"dataset", VDV_STATUS, IFERROR(FILTER(VDV_B, VDV_A="gdp"), ""))</f>
         <v/>
       </c>
-      <c r="B6">
+      <c r="B6" s="30">
         <f>IFERROR(FILTER(VDV_C, VDV_A="gdp"), "")</f>
         <v/>
       </c>
@@ -828,7 +842,7 @@
         <f>IFERROR(ARRAYFORMULA(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(FILTER(VDV_D, VDV_A="gdp"), "agriculture", "Nông-lâm-thủy sản"), "industry", "Công nghiệp-xây dựng"), "services", "Dịch vụ"), "total", "Toàn nền kinh tế")), "")</f>
         <v/>
       </c>
-      <c r="D6">
+      <c r="D6" s="27">
         <f>IFERROR(FILTER(VDV_F, VDV_A="gdp"), "")</f>
         <v/>
       </c>
@@ -918,23 +932,23 @@
         <f>IF(VDV_STATUS&lt;&gt;"dataset", VDV_STATUS, IFERROR(ARRAYFORMULA(TEXT(FILTER(VDV_B, VDV_A="trade"), "yyyy-mm")), ""))</f>
         <v/>
       </c>
-      <c r="B6">
+      <c r="B6" s="27">
         <f>IFERROR(FILTER(VDV_C, VDV_A="trade"), "")</f>
         <v/>
       </c>
-      <c r="C6">
+      <c r="C6" s="27">
         <f>IFERROR(FILTER(VDV_D, VDV_A="trade"), "")</f>
         <v/>
       </c>
-      <c r="D6">
+      <c r="D6" s="27">
         <f>IFERROR(FILTER(VDV_E, VDV_A="trade"), "")</f>
         <v/>
       </c>
-      <c r="E6">
+      <c r="E6" s="32">
         <f>IFERROR(FILTER(VDV_F, VDV_A="trade"), "")</f>
         <v/>
       </c>
-      <c r="F6">
+      <c r="F6" s="32">
         <f>IFERROR(FILTER(VDV_G, VDV_A="trade"), "")</f>
         <v/>
       </c>
@@ -1782,11 +1796,11 @@
         <f>IF(VDV_STATUS&lt;&gt;"dataset", VDV_STATUS, IFERROR(ARRAYFORMULA(TEXT(FILTER(VDV_B, VDV_A="gold"), "yyyy-mm-dd")), ""))</f>
         <v/>
       </c>
-      <c r="B6">
+      <c r="B6" s="23">
         <f>IFERROR(FILTER(VDV_C, VDV_A="gold"), "")</f>
         <v/>
       </c>
-      <c r="C6">
+      <c r="C6" s="23">
         <f>IFERROR(FILTER(VDV_D, VDV_A="gold"), "")</f>
         <v/>
       </c>
@@ -1850,11 +1864,11 @@
         <f>IF(VDV_STATUS&lt;&gt;"dataset", VDV_STATUS, IFERROR(ARRAYFORMULA(TEXT(FILTER(VDV_B, VDV_A="silver"), "yyyy-mm-dd")), ""))</f>
         <v/>
       </c>
-      <c r="B6">
+      <c r="B6" s="23">
         <f>IFERROR(FILTER(VDV_C, VDV_A="silver"), "")</f>
         <v/>
       </c>
-      <c r="C6">
+      <c r="C6" s="23">
         <f>IFERROR(FILTER(VDV_D, VDV_A="silver"), "")</f>
         <v/>
       </c>
@@ -1948,31 +1962,31 @@
         <f>IF(VDV_STATUS&lt;&gt;"dataset", VDV_STATUS, IFERROR(ARRAYFORMULA(TEXT(FILTER(VDV_B, VDV_A="interbank"), "yyyy-mm-dd")), ""))</f>
         <v/>
       </c>
-      <c r="B6">
+      <c r="B6" s="27">
         <f>IFERROR(FILTER(VDV_C, VDV_A="interbank"), "")</f>
         <v/>
       </c>
-      <c r="C6">
+      <c r="C6" s="27">
         <f>IFERROR(FILTER(VDV_D, VDV_A="interbank"), "")</f>
         <v/>
       </c>
-      <c r="D6">
+      <c r="D6" s="27">
         <f>IFERROR(FILTER(VDV_E, VDV_A="interbank"), "")</f>
         <v/>
       </c>
-      <c r="E6">
+      <c r="E6" s="27">
         <f>IFERROR(FILTER(VDV_F, VDV_A="interbank"), "")</f>
         <v/>
       </c>
-      <c r="F6">
+      <c r="F6" s="27">
         <f>IFERROR(FILTER(VDV_G, VDV_A="interbank"), "")</f>
         <v/>
       </c>
-      <c r="G6">
+      <c r="G6" s="27">
         <f>IFERROR(FILTER(VDV_H, VDV_A="interbank"), "")</f>
         <v/>
       </c>
-      <c r="H6">
+      <c r="H6" s="27">
         <f>IFERROR(FILTER(VDV_I, VDV_A="interbank"), "")</f>
         <v/>
       </c>
@@ -2030,7 +2044,7 @@
         <f>IF(VDV_STATUS&lt;&gt;"dataset", VDV_STATUS, IFERROR(ARRAYFORMULA(TEXT(FILTER(VDV_B, VDV_A="fx"), "yyyy-mm-dd")), ""))</f>
         <v/>
       </c>
-      <c r="B6">
+      <c r="B6" s="23">
         <f>IFERROR(FILTER(VDV_C, VDV_A="fx"), "")</f>
         <v/>
       </c>
@@ -2112,23 +2126,23 @@
         <f>IF(VDV_STATUS&lt;&gt;"dataset", VDV_STATUS, IFERROR(ARRAYFORMULA(TEXT(FILTER(VDV_B, VDV_A="deposit"), "yyyy-mm-dd")), ""))</f>
         <v/>
       </c>
-      <c r="B6">
+      <c r="B6" s="27">
         <f>IFERROR(FILTER(VDV_C, VDV_A="deposit"), "")</f>
         <v/>
       </c>
-      <c r="C6">
+      <c r="C6" s="27">
         <f>IFERROR(FILTER(VDV_D, VDV_A="deposit"), "")</f>
         <v/>
       </c>
-      <c r="D6">
+      <c r="D6" s="27">
         <f>IFERROR(FILTER(VDV_E, VDV_A="deposit"), "")</f>
         <v/>
       </c>
-      <c r="E6">
+      <c r="E6" s="27">
         <f>IFERROR(FILTER(VDV_F, VDV_A="deposit"), "")</f>
         <v/>
       </c>
-      <c r="F6">
+      <c r="F6" s="27">
         <f>IFERROR(FILTER(VDV_G, VDV_A="deposit"), "")</f>
         <v/>
       </c>
@@ -2198,15 +2212,15 @@
         <f>IF(VDV_STATUS&lt;&gt;"dataset", VDV_STATUS, IFERROR(ARRAYFORMULA(TEXT(FILTER(VDV_B, VDV_A="global"), "yyyy-mm-dd")), ""))</f>
         <v/>
       </c>
-      <c r="B6">
+      <c r="B6" s="28">
         <f>IFERROR(FILTER(VDV_C, VDV_A="global"), "")</f>
         <v/>
       </c>
-      <c r="C6">
+      <c r="C6" s="29">
         <f>IFERROR(FILTER(VDV_D, VDV_A="global"), "")</f>
         <v/>
       </c>
-      <c r="D6">
+      <c r="D6" s="23">
         <f>IFERROR(FILTER(VDV_E, VDV_A="global"), "")</f>
         <v/>
       </c>
@@ -2270,11 +2284,11 @@
         <f>IF(VDV_STATUS&lt;&gt;"dataset", VDV_STATUS, IFERROR(ARRAYFORMULA(TEXT(FILTER(VDV_B, VDV_A="cpi"), "yyyy-mm")), ""))</f>
         <v/>
       </c>
-      <c r="B6">
+      <c r="B6" s="27">
         <f>IFERROR(FILTER(VDV_C, VDV_A="cpi"), "")</f>
         <v/>
       </c>
-      <c r="C6">
+      <c r="C6" s="27">
         <f>IFERROR(FILTER(VDV_D, VDV_A="cpi"), "")</f>
         <v/>
       </c>

</xml_diff>